<commit_message>
Add responsive title page variant
</commit_message>
<xml_diff>
--- a/Расчет_список.xlsx
+++ b/Расчет_список.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Roman\Documents\DD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15D19B0B-CEC7-40AE-B226-6DEBA1E0396A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF4F1D7B-CA05-4A82-A362-B7B8665FA946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A77F7C32-41CE-594D-B64E-396197F2C882}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,6 +27,7 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -196,9 +197,6 @@
     <t>Дети</t>
   </si>
   <si>
-    <t>Молодеж</t>
-  </si>
-  <si>
     <t>Рабочий возраст</t>
   </si>
   <si>
@@ -284,15 +282,15 @@
   </si>
   <si>
     <t>SberPay Вжух</t>
+  </si>
+  <si>
+    <t>Молодежь</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -375,7 +373,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -383,14 +381,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -710,6 +711,7 @@
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="47.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" style="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -720,7 +722,7 @@
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="9" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
@@ -738,15 +740,15 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D2" s="3">
+        <v>78</v>
+      </c>
+      <c r="D2" s="10">
         <v>0.62574257425742574</v>
       </c>
       <c r="E2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -760,13 +762,13 @@
       <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="10">
         <v>0.62574257425742574</v>
       </c>
       <c r="E3" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -780,13 +782,13 @@
       <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="10">
         <v>0.47640449438202248</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -800,13 +802,13 @@
       <c r="C5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5" s="10">
         <v>0.41396508728179554</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -820,13 +822,13 @@
       <c r="C6" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="10">
         <v>0.36082474226804123</v>
       </c>
       <c r="E6" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -840,13 +842,13 @@
       <c r="C7" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7" s="10">
         <v>0.46419753086419757</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -860,13 +862,13 @@
       <c r="C8" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8" s="10">
         <v>0.46236559139784944</v>
       </c>
       <c r="E8" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -880,13 +882,13 @@
       <c r="C9" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9" s="10">
         <v>0.39999999999999997</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -900,13 +902,13 @@
       <c r="C10" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10" s="10">
         <v>0.44158415841584159</v>
       </c>
       <c r="E10" t="s">
         <v>10</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -920,13 +922,13 @@
       <c r="C11" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11" s="10">
         <v>0.47010309278350515</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -940,13 +942,13 @@
       <c r="C12" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="10">
         <v>0.63505154639175254</v>
       </c>
       <c r="E12" t="s">
         <v>6</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="F12" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -960,13 +962,13 @@
       <c r="C13" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13" s="10">
         <v>0.53195876288659794</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="F13" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -980,13 +982,13 @@
       <c r="C14" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="10">
         <v>0.60990099009900989</v>
       </c>
       <c r="E14" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1000,13 +1002,13 @@
       <c r="C15" t="s">
         <v>22</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="10">
         <v>0.57029702970297036</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="F15" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1020,13 +1022,13 @@
       <c r="C16" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="10">
         <v>0.38651685393258428</v>
       </c>
       <c r="E16" t="s">
         <v>13</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1040,13 +1042,13 @@
       <c r="C17" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="10">
         <v>0.51546391752577314</v>
       </c>
       <c r="E17" t="s">
         <v>10</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="F17" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1060,13 +1062,13 @@
       <c r="C18" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18" s="10">
         <v>0.59381443298969061</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="F18" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1080,13 +1082,13 @@
       <c r="C19" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19" s="10">
         <v>0.54491017964071853</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="F19" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1100,13 +1102,13 @@
       <c r="C20" t="s">
         <v>27</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="10">
         <v>0.5388235294117647</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1120,13 +1122,13 @@
       <c r="C21" t="s">
         <v>28</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21" s="10">
         <v>0.55730337078651682</v>
       </c>
       <c r="E21" t="s">
         <v>10</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="F21" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1140,13 +1142,13 @@
       <c r="C22" t="s">
         <v>29</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22" s="10">
         <v>0.2880886426592798</v>
       </c>
       <c r="E22" t="s">
         <v>13</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1160,13 +1162,13 @@
       <c r="C23" t="s">
         <v>31</v>
       </c>
-      <c r="D23" s="3">
+      <c r="D23" s="10">
         <v>0.33980582524271846</v>
       </c>
       <c r="E23" t="s">
         <v>13</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="F23" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1180,13 +1182,13 @@
       <c r="C24" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="3">
+      <c r="D24" s="10">
         <v>0.60759493670886078</v>
       </c>
       <c r="E24" t="s">
         <v>6</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="F24" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1200,13 +1202,13 @@
       <c r="C25" t="s">
         <v>33</v>
       </c>
-      <c r="D25" s="3">
+      <c r="D25" s="10">
         <v>0.55089820359281438</v>
       </c>
       <c r="E25" t="s">
         <v>10</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="F25" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1220,13 +1222,13 @@
       <c r="C26" t="s">
         <v>34</v>
       </c>
-      <c r="D26" s="3">
+      <c r="D26" s="10">
         <v>0.47524752475247523</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1240,13 +1242,13 @@
       <c r="C27" t="s">
         <v>35</v>
       </c>
-      <c r="D27" s="3">
+      <c r="D27" s="10">
         <v>0.55172413793103448</v>
       </c>
       <c r="E27" t="s">
         <v>10</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="F27" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1260,13 +1262,13 @@
       <c r="C28" t="s">
         <v>36</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D28" s="10">
         <v>0.5544554455445545</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1277,16 +1279,16 @@
       <c r="B29" t="s">
         <v>30</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="D29" s="3">
+      <c r="D29" s="10">
         <v>0.28817204301075267</v>
       </c>
       <c r="E29" t="s">
         <v>13</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="F29" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1300,13 +1302,13 @@
       <c r="C30" t="s">
         <v>38</v>
       </c>
-      <c r="D30" s="3">
+      <c r="D30" s="10">
         <v>0.76831683168316822</v>
       </c>
       <c r="E30" t="s">
         <v>6</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="F30" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1320,13 +1322,13 @@
       <c r="C31" t="s">
         <v>39</v>
       </c>
-      <c r="D31" s="3">
+      <c r="D31" s="10">
         <v>0.3827956989247312</v>
       </c>
       <c r="E31" t="s">
         <v>13</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="F31" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1340,13 +1342,13 @@
       <c r="C32" t="s">
         <v>40</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D32" s="10">
         <v>0.34408602150537637</v>
       </c>
       <c r="E32" t="s">
         <v>13</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="F32" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1357,16 +1359,16 @@
       <c r="B33" t="s">
         <v>41</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D33" s="3">
+      <c r="D33" s="10">
         <v>0.67010309278350511</v>
       </c>
       <c r="E33" t="s">
         <v>6</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="F33" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1380,13 +1382,13 @@
       <c r="C34" t="s">
         <v>43</v>
       </c>
-      <c r="D34" s="3">
+      <c r="D34" s="10">
         <v>0.6</v>
       </c>
       <c r="E34" t="s">
         <v>6</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="F34" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1400,13 +1402,13 @@
       <c r="C35" t="s">
         <v>44</v>
       </c>
-      <c r="D35" s="3">
+      <c r="D35" s="10">
         <v>0.73267326732673266</v>
       </c>
       <c r="E35" t="s">
         <v>6</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="F35" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1420,13 +1422,13 @@
       <c r="C36" t="s">
         <v>46</v>
       </c>
-      <c r="D36" s="3">
+      <c r="D36" s="10">
         <v>0.52861952861952854</v>
       </c>
       <c r="E36" t="s">
         <v>10</v>
       </c>
-      <c r="F36" s="6" t="s">
+      <c r="F36" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1434,19 +1436,19 @@
       <c r="A37">
         <v>229</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B37" s="3" t="s">
         <v>47</v>
       </c>
       <c r="C37" t="s">
         <v>48</v>
       </c>
-      <c r="D37" s="3">
+      <c r="D37" s="10">
         <v>0.57731958762886593</v>
       </c>
       <c r="E37" t="s">
         <v>10</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="F37" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1454,19 +1456,19 @@
       <c r="A38">
         <v>234</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="3" t="s">
         <v>47</v>
       </c>
       <c r="C38" t="s">
         <v>49</v>
       </c>
-      <c r="D38" s="3">
+      <c r="D38" s="10">
         <v>0.56831683168316827</v>
       </c>
       <c r="E38" t="s">
         <v>10</v>
       </c>
-      <c r="F38" s="4" t="s">
+      <c r="F38" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1474,179 +1476,179 @@
       <c r="A39">
         <v>239</v>
       </c>
-      <c r="B39" s="4" t="s">
+      <c r="B39" s="3" t="s">
         <v>47</v>
       </c>
       <c r="C39" t="s">
         <v>50</v>
       </c>
-      <c r="D39" s="3">
+      <c r="D39" s="10">
         <v>0.44950495049504952</v>
       </c>
       <c r="E39" t="s">
         <v>10</v>
       </c>
-      <c r="F39" s="4" t="s">
+      <c r="F39" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="7">
+      <c r="A40" s="6">
         <v>13</v>
       </c>
-      <c r="B40" s="8" t="s">
+      <c r="B40" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="C40" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D40" s="9">
+      <c r="D40" s="11">
         <v>0.58397932816537468</v>
       </c>
-      <c r="E40" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F40" s="8" t="s">
-        <v>80</v>
+      <c r="E40" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="7">
+      <c r="A41" s="6">
         <v>18</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B41" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="D41" s="11">
+        <v>0.53180661577608146</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="6">
+        <v>23</v>
+      </c>
+      <c r="B42" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C42" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="9">
-        <v>0.53180661577608146</v>
-      </c>
-      <c r="E41" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F41" s="8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="7">
-        <v>23</v>
-      </c>
-      <c r="B42" s="8" t="s">
+      <c r="D42" s="11">
+        <v>0.67153284671532842</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="6">
+        <v>28</v>
+      </c>
+      <c r="B43" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C43" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D42" s="9">
-        <v>0.67153284671532842</v>
-      </c>
-      <c r="E42" s="7" t="s">
+      <c r="D43" s="11">
+        <v>0.49109414758269726</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="6">
+        <v>33</v>
+      </c>
+      <c r="B44" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="D44" s="11">
+        <v>0.59890109890109888</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="6">
+        <v>38</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D45" s="11">
+        <v>0.6797752808988764</v>
+      </c>
+      <c r="E45" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F42" s="8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="7">
-        <v>28</v>
-      </c>
-      <c r="B43" s="8" t="s">
+      <c r="F45" s="7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="6">
+        <v>43</v>
+      </c>
+      <c r="B46" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C43" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="D43" s="9">
-        <v>0.49109414758269726</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F43" s="8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="7">
-        <v>33</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C44" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="D44" s="9">
-        <v>0.59890109890109888</v>
-      </c>
-      <c r="E44" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F44" s="8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="7">
-        <v>38</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C45" s="10" t="s">
+      <c r="C46" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="D45" s="9">
-        <v>0.6797752808988764</v>
-      </c>
-      <c r="E45" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="F45" s="8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="7">
-        <v>43</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C46" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="D46" s="9">
+      <c r="D46" s="11">
         <v>0.4438202247191011</v>
       </c>
-      <c r="E46" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F46" s="8" t="s">
-        <v>80</v>
+      <c r="E46" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>260</v>
       </c>
-      <c r="B47" s="4" t="s">
+      <c r="B47" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C47" t="s">
         <v>58</v>
       </c>
-      <c r="C47" t="s">
-        <v>59</v>
-      </c>
-      <c r="D47" s="3">
+      <c r="D47" s="10">
         <v>0.34457831325301208</v>
       </c>
       <c r="E47" t="s">
         <v>13</v>
       </c>
-      <c r="F47" s="4" t="s">
+      <c r="F47" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1654,19 +1656,19 @@
       <c r="A48">
         <v>280</v>
       </c>
-      <c r="B48" s="4" t="s">
-        <v>58</v>
+      <c r="B48" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C48" t="s">
-        <v>60</v>
-      </c>
-      <c r="D48" s="3">
+        <v>59</v>
+      </c>
+      <c r="D48" s="10">
         <v>0.27586206896551724</v>
       </c>
       <c r="E48" t="s">
         <v>13</v>
       </c>
-      <c r="F48" s="4" t="s">
+      <c r="F48" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1674,19 +1676,19 @@
       <c r="A49">
         <v>285</v>
       </c>
-      <c r="B49" s="4" t="s">
-        <v>58</v>
+      <c r="B49" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C49" t="s">
-        <v>61</v>
-      </c>
-      <c r="D49" s="3">
+        <v>60</v>
+      </c>
+      <c r="D49" s="10">
         <v>0.24</v>
       </c>
       <c r="E49" t="s">
         <v>13</v>
       </c>
-      <c r="F49" s="4" t="s">
+      <c r="F49" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1694,19 +1696,19 @@
       <c r="A50">
         <v>290</v>
       </c>
-      <c r="B50" s="4" t="s">
-        <v>58</v>
+      <c r="B50" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C50" t="s">
-        <v>62</v>
-      </c>
-      <c r="D50" s="3">
+        <v>61</v>
+      </c>
+      <c r="D50" s="10">
         <v>0.35632183908045978</v>
       </c>
       <c r="E50" t="s">
         <v>13</v>
       </c>
-      <c r="F50" s="4" t="s">
+      <c r="F50" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1714,19 +1716,19 @@
       <c r="A51">
         <v>300</v>
       </c>
-      <c r="B51" s="4" t="s">
-        <v>58</v>
+      <c r="B51" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C51" t="s">
-        <v>63</v>
-      </c>
-      <c r="D51" s="3">
+        <v>62</v>
+      </c>
+      <c r="D51" s="10">
         <v>0.58969072164948455</v>
       </c>
       <c r="E51" t="s">
         <v>10</v>
       </c>
-      <c r="F51" s="4" t="s">
+      <c r="F51" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1734,19 +1736,19 @@
       <c r="A52">
         <v>315</v>
       </c>
-      <c r="B52" s="4" t="s">
-        <v>58</v>
+      <c r="B52" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C52" t="s">
-        <v>64</v>
-      </c>
-      <c r="D52" s="3">
+        <v>63</v>
+      </c>
+      <c r="D52" s="10">
         <v>0.37362637362637363</v>
       </c>
       <c r="E52" t="s">
         <v>13</v>
       </c>
-      <c r="F52" s="4" t="s">
+      <c r="F52" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1754,19 +1756,19 @@
       <c r="A53">
         <v>320</v>
       </c>
-      <c r="B53" s="4" t="s">
-        <v>58</v>
+      <c r="B53" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C53" t="s">
-        <v>65</v>
-      </c>
-      <c r="D53" s="3">
+        <v>64</v>
+      </c>
+      <c r="D53" s="10">
         <v>0.36831683168316837</v>
       </c>
       <c r="E53" t="s">
         <v>13</v>
       </c>
-      <c r="F53" s="4" t="s">
+      <c r="F53" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1774,19 +1776,19 @@
       <c r="A54">
         <v>325</v>
       </c>
-      <c r="B54" s="4" t="s">
-        <v>58</v>
+      <c r="B54" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C54" t="s">
-        <v>66</v>
-      </c>
-      <c r="D54" s="3">
+        <v>65</v>
+      </c>
+      <c r="D54" s="10">
         <v>0.68247422680412373</v>
       </c>
       <c r="E54" t="s">
         <v>6</v>
       </c>
-      <c r="F54" s="4" t="s">
+      <c r="F54" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1794,19 +1796,19 @@
       <c r="A55">
         <v>330</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>58</v>
+      <c r="B55" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C55" t="s">
-        <v>67</v>
-      </c>
-      <c r="D55" s="3">
+        <v>66</v>
+      </c>
+      <c r="D55" s="10">
         <v>0.37354988399071926</v>
       </c>
       <c r="E55" t="s">
         <v>13</v>
       </c>
-      <c r="F55" s="4" t="s">
+      <c r="F55" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1814,19 +1816,19 @@
       <c r="A56">
         <v>335</v>
       </c>
-      <c r="B56" s="4" t="s">
-        <v>58</v>
+      <c r="B56" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C56" t="s">
-        <v>68</v>
-      </c>
-      <c r="D56" s="3">
+        <v>67</v>
+      </c>
+      <c r="D56" s="10">
         <v>0.65822784810126578</v>
       </c>
       <c r="E56" t="s">
         <v>6</v>
       </c>
-      <c r="F56" s="4" t="s">
+      <c r="F56" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1834,19 +1836,19 @@
       <c r="A57">
         <v>340</v>
       </c>
-      <c r="B57" s="4" t="s">
-        <v>58</v>
+      <c r="B57" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C57" t="s">
-        <v>69</v>
-      </c>
-      <c r="D57" s="3">
+        <v>68</v>
+      </c>
+      <c r="D57" s="10">
         <v>0.62650602409638556</v>
       </c>
       <c r="E57" t="s">
         <v>6</v>
       </c>
-      <c r="F57" s="4" t="s">
+      <c r="F57" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1854,19 +1856,19 @@
       <c r="A58">
         <v>345</v>
       </c>
-      <c r="B58" s="4" t="s">
-        <v>58</v>
+      <c r="B58" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C58" t="s">
-        <v>70</v>
-      </c>
-      <c r="D58" s="3">
+        <v>69</v>
+      </c>
+      <c r="D58" s="10">
         <v>0.55643564356435649</v>
       </c>
       <c r="E58" t="s">
         <v>10</v>
       </c>
-      <c r="F58" s="4" t="s">
+      <c r="F58" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1874,19 +1876,19 @@
       <c r="A59">
         <v>350</v>
       </c>
-      <c r="B59" s="4" t="s">
-        <v>58</v>
+      <c r="B59" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C59" t="s">
-        <v>71</v>
-      </c>
-      <c r="D59" s="3">
+        <v>70</v>
+      </c>
+      <c r="D59" s="10">
         <v>0.77367205542725181</v>
       </c>
       <c r="E59" t="s">
         <v>6</v>
       </c>
-      <c r="F59" s="4" t="s">
+      <c r="F59" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1894,19 +1896,19 @@
       <c r="A60">
         <v>355</v>
       </c>
-      <c r="B60" s="4" t="s">
-        <v>58</v>
+      <c r="B60" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C60" t="s">
-        <v>72</v>
-      </c>
-      <c r="D60" s="3">
+        <v>71</v>
+      </c>
+      <c r="D60" s="10">
         <v>0.36263736263736263</v>
       </c>
       <c r="E60" t="s">
         <v>13</v>
       </c>
-      <c r="F60" s="4" t="s">
+      <c r="F60" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1914,19 +1916,19 @@
       <c r="A61">
         <v>360</v>
       </c>
-      <c r="B61" s="4" t="s">
-        <v>58</v>
+      <c r="B61" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C61" t="s">
-        <v>65</v>
-      </c>
-      <c r="D61" s="3">
+        <v>64</v>
+      </c>
+      <c r="D61" s="10">
         <v>0.45940594059405937</v>
       </c>
       <c r="E61" t="s">
         <v>10</v>
       </c>
-      <c r="F61" s="4" t="s">
+      <c r="F61" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1934,19 +1936,19 @@
       <c r="A62">
         <v>365</v>
       </c>
-      <c r="B62" s="4" t="s">
-        <v>58</v>
+      <c r="B62" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C62" t="s">
-        <v>73</v>
-      </c>
-      <c r="D62" s="3">
+        <v>72</v>
+      </c>
+      <c r="D62" s="10">
         <v>0.37349397590361444</v>
       </c>
       <c r="E62" t="s">
         <v>13</v>
       </c>
-      <c r="F62" s="4" t="s">
+      <c r="F62" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1954,19 +1956,19 @@
       <c r="A63">
         <v>370</v>
       </c>
-      <c r="B63" s="4" t="s">
-        <v>58</v>
+      <c r="B63" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C63" t="s">
-        <v>74</v>
-      </c>
-      <c r="D63" s="3">
+        <v>73</v>
+      </c>
+      <c r="D63" s="10">
         <v>0.41445783132530117</v>
       </c>
       <c r="E63" t="s">
         <v>10</v>
       </c>
-      <c r="F63" s="4" t="s">
+      <c r="F63" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1974,19 +1976,19 @@
       <c r="A64">
         <v>375</v>
       </c>
-      <c r="B64" s="4" t="s">
-        <v>58</v>
+      <c r="B64" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C64" t="s">
-        <v>81</v>
-      </c>
-      <c r="D64" s="3">
+        <v>80</v>
+      </c>
+      <c r="D64" s="10">
         <v>0.4206896551724138</v>
       </c>
       <c r="E64" t="s">
         <v>10</v>
       </c>
-      <c r="F64" s="4" t="s">
+      <c r="F64" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1994,19 +1996,19 @@
       <c r="A65">
         <v>380</v>
       </c>
-      <c r="B65" s="4" t="s">
-        <v>58</v>
+      <c r="B65" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C65" t="s">
-        <v>75</v>
-      </c>
-      <c r="D65" s="3">
+        <v>74</v>
+      </c>
+      <c r="D65" s="10">
         <v>0.33195876288659798</v>
       </c>
       <c r="E65" t="s">
         <v>13</v>
       </c>
-      <c r="F65" s="4" t="s">
+      <c r="F65" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2014,19 +2016,19 @@
       <c r="A66">
         <v>390</v>
       </c>
-      <c r="B66" s="4" t="s">
-        <v>58</v>
+      <c r="B66" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C66" t="s">
-        <v>76</v>
-      </c>
-      <c r="D66" s="3">
+        <v>75</v>
+      </c>
+      <c r="D66" s="10">
         <v>0.3935483870967742</v>
       </c>
       <c r="E66" t="s">
         <v>13</v>
       </c>
-      <c r="F66" s="4" t="s">
+      <c r="F66" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2034,19 +2036,19 @@
       <c r="A67">
         <v>405</v>
       </c>
-      <c r="B67" s="4" t="s">
-        <v>58</v>
+      <c r="B67" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C67" t="s">
-        <v>77</v>
-      </c>
-      <c r="D67" s="3">
+        <v>76</v>
+      </c>
+      <c r="D67" s="10">
         <v>0.33806146572104023</v>
       </c>
       <c r="E67" t="s">
         <v>13</v>
       </c>
-      <c r="F67" s="4" t="s">
+      <c r="F67" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2054,346 +2056,342 @@
       <c r="A68">
         <v>410</v>
       </c>
-      <c r="B68" s="4" t="s">
-        <v>58</v>
+      <c r="B68" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C68" t="s">
-        <v>78</v>
-      </c>
-      <c r="D68" s="3">
+        <v>77</v>
+      </c>
+      <c r="D68" s="10">
         <v>0.39958592132505177</v>
       </c>
       <c r="E68" t="s">
         <v>13</v>
       </c>
-      <c r="F68" s="4" t="s">
+      <c r="F68" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B69" s="4"/>
-      <c r="D69" s="3"/>
+      <c r="B69" s="3"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B70" s="4"/>
-      <c r="D70" s="3"/>
+      <c r="B70" s="3"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B71" s="4"/>
-      <c r="D71" s="3"/>
+      <c r="B71" s="3"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B72" s="4"/>
-      <c r="D72" s="3"/>
+      <c r="B72" s="3"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B73" s="4"/>
+      <c r="B73" s="3"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B74" s="4"/>
+      <c r="B74" s="3"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B75" s="4"/>
+      <c r="B75" s="3"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B76" s="4"/>
+      <c r="B76" s="3"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B77" s="4"/>
+      <c r="B77" s="3"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B78" s="4"/>
+      <c r="B78" s="3"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B79" s="4"/>
+      <c r="B79" s="3"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B80" s="4"/>
+      <c r="B80" s="3"/>
     </row>
     <row r="81" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B81" s="4"/>
+      <c r="B81" s="3"/>
     </row>
     <row r="82" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B82" s="4"/>
+      <c r="B82" s="3"/>
     </row>
     <row r="83" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B83" s="4"/>
+      <c r="B83" s="3"/>
     </row>
     <row r="84" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B84" s="4"/>
+      <c r="B84" s="3"/>
     </row>
     <row r="85" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B85" s="4"/>
+      <c r="B85" s="3"/>
     </row>
     <row r="86" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B86" s="4"/>
+      <c r="B86" s="3"/>
     </row>
     <row r="87" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B87" s="4"/>
+      <c r="B87" s="3"/>
     </row>
     <row r="88" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B88" s="4"/>
+      <c r="B88" s="3"/>
     </row>
     <row r="89" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B89" s="4"/>
+      <c r="B89" s="3"/>
     </row>
     <row r="90" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B90" s="4"/>
+      <c r="B90" s="3"/>
     </row>
     <row r="91" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B91" s="4"/>
+      <c r="B91" s="3"/>
     </row>
     <row r="92" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B92" s="4"/>
+      <c r="B92" s="3"/>
     </row>
     <row r="93" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B93" s="4"/>
+      <c r="B93" s="3"/>
     </row>
     <row r="94" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B94" s="4"/>
+      <c r="B94" s="3"/>
     </row>
     <row r="95" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B95" s="4"/>
+      <c r="B95" s="3"/>
     </row>
     <row r="96" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B96" s="4"/>
+      <c r="B96" s="3"/>
     </row>
     <row r="97" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B97" s="4"/>
+      <c r="B97" s="3"/>
     </row>
     <row r="98" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B98" s="4"/>
+      <c r="B98" s="3"/>
     </row>
     <row r="99" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B99" s="4"/>
+      <c r="B99" s="3"/>
     </row>
     <row r="100" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B100" s="4"/>
+      <c r="B100" s="3"/>
     </row>
     <row r="101" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B101" s="4"/>
+      <c r="B101" s="3"/>
     </row>
     <row r="102" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B102" s="4"/>
+      <c r="B102" s="3"/>
     </row>
     <row r="103" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B103" s="4"/>
+      <c r="B103" s="3"/>
     </row>
     <row r="104" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B104" s="4"/>
+      <c r="B104" s="3"/>
     </row>
     <row r="105" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B105" s="4"/>
+      <c r="B105" s="3"/>
     </row>
     <row r="106" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B106" s="4"/>
+      <c r="B106" s="3"/>
     </row>
     <row r="107" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B107" s="4"/>
+      <c r="B107" s="3"/>
     </row>
     <row r="108" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B108" s="4"/>
+      <c r="B108" s="3"/>
     </row>
     <row r="109" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B109" s="4"/>
+      <c r="B109" s="3"/>
     </row>
     <row r="110" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B110" s="4"/>
+      <c r="B110" s="3"/>
     </row>
     <row r="111" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B111" s="4"/>
+      <c r="B111" s="3"/>
     </row>
     <row r="112" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B112" s="4"/>
+      <c r="B112" s="3"/>
     </row>
     <row r="113" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B113" s="4"/>
+      <c r="B113" s="3"/>
     </row>
     <row r="114" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B114" s="4"/>
+      <c r="B114" s="3"/>
     </row>
     <row r="115" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B115" s="4"/>
+      <c r="B115" s="3"/>
     </row>
     <row r="116" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B116" s="4"/>
+      <c r="B116" s="3"/>
     </row>
     <row r="117" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B117" s="4"/>
+      <c r="B117" s="3"/>
     </row>
     <row r="118" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B118" s="4"/>
+      <c r="B118" s="3"/>
     </row>
     <row r="119" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B119" s="4"/>
+      <c r="B119" s="3"/>
     </row>
     <row r="120" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B120" s="4"/>
+      <c r="B120" s="3"/>
     </row>
     <row r="121" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B121" s="4"/>
+      <c r="B121" s="3"/>
     </row>
     <row r="122" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B122" s="4"/>
+      <c r="B122" s="3"/>
     </row>
     <row r="123" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B123" s="4"/>
+      <c r="B123" s="3"/>
     </row>
     <row r="124" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B124" s="4"/>
+      <c r="B124" s="3"/>
     </row>
     <row r="125" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B125" s="4"/>
+      <c r="B125" s="3"/>
     </row>
     <row r="126" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B126" s="4"/>
+      <c r="B126" s="3"/>
     </row>
     <row r="127" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B127" s="4"/>
+      <c r="B127" s="3"/>
     </row>
     <row r="128" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B128" s="4"/>
+      <c r="B128" s="3"/>
     </row>
     <row r="129" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B129" s="4"/>
+      <c r="B129" s="3"/>
     </row>
     <row r="130" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B130" s="4"/>
+      <c r="B130" s="3"/>
     </row>
     <row r="131" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B131" s="4"/>
+      <c r="B131" s="3"/>
     </row>
     <row r="132" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B132" s="4"/>
+      <c r="B132" s="3"/>
     </row>
     <row r="133" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B133" s="4"/>
+      <c r="B133" s="3"/>
     </row>
     <row r="134" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B134" s="4"/>
+      <c r="B134" s="3"/>
     </row>
     <row r="135" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B135" s="4"/>
+      <c r="B135" s="3"/>
     </row>
     <row r="136" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B136" s="4"/>
+      <c r="B136" s="3"/>
     </row>
     <row r="137" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B137" s="4"/>
+      <c r="B137" s="3"/>
     </row>
     <row r="138" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B138" s="4"/>
+      <c r="B138" s="3"/>
     </row>
     <row r="139" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B139" s="4"/>
+      <c r="B139" s="3"/>
     </row>
     <row r="140" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B140" s="4"/>
+      <c r="B140" s="3"/>
     </row>
     <row r="141" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B141" s="4"/>
+      <c r="B141" s="3"/>
     </row>
     <row r="142" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B142" s="4"/>
+      <c r="B142" s="3"/>
     </row>
     <row r="143" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B143" s="4"/>
+      <c r="B143" s="3"/>
     </row>
     <row r="144" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B144" s="4"/>
+      <c r="B144" s="3"/>
     </row>
     <row r="145" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B145" s="4"/>
+      <c r="B145" s="3"/>
     </row>
     <row r="146" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B146" s="4"/>
+      <c r="B146" s="3"/>
     </row>
     <row r="147" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B147" s="4"/>
+      <c r="B147" s="3"/>
     </row>
     <row r="148" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B148" s="4"/>
+      <c r="B148" s="3"/>
     </row>
     <row r="149" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B149" s="4"/>
+      <c r="B149" s="3"/>
     </row>
     <row r="150" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B150" s="4"/>
+      <c r="B150" s="3"/>
     </row>
     <row r="151" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B151" s="4"/>
+      <c r="B151" s="3"/>
     </row>
     <row r="152" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B152" s="4"/>
+      <c r="B152" s="3"/>
     </row>
     <row r="153" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B153" s="4"/>
+      <c r="B153" s="3"/>
     </row>
     <row r="154" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B154" s="4"/>
+      <c r="B154" s="3"/>
     </row>
     <row r="155" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B155" s="4"/>
+      <c r="B155" s="3"/>
     </row>
     <row r="156" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B156" s="4"/>
+      <c r="B156" s="3"/>
     </row>
     <row r="157" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B157" s="4"/>
+      <c r="B157" s="3"/>
     </row>
     <row r="158" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B158" s="4"/>
+      <c r="B158" s="3"/>
     </row>
     <row r="159" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B159" s="4"/>
+      <c r="B159" s="3"/>
     </row>
     <row r="160" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B160" s="4"/>
+      <c r="B160" s="3"/>
     </row>
     <row r="161" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B161" s="4"/>
+      <c r="B161" s="3"/>
     </row>
     <row r="162" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B162" s="4"/>
+      <c r="B162" s="3"/>
     </row>
     <row r="163" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B163" s="4"/>
+      <c r="B163" s="3"/>
     </row>
     <row r="164" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B164" s="4"/>
+      <c r="B164" s="3"/>
     </row>
     <row r="165" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B165" s="4"/>
+      <c r="B165" s="3"/>
     </row>
     <row r="166" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B166" s="4"/>
+      <c r="B166" s="3"/>
     </row>
     <row r="167" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B167" s="4"/>
+      <c r="B167" s="3"/>
     </row>
     <row r="168" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B168" s="4"/>
+      <c r="B168" s="3"/>
     </row>
     <row r="169" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B169" s="4"/>
+      <c r="B169" s="3"/>
     </row>
     <row r="170" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B170" s="4"/>
+      <c r="B170" s="3"/>
     </row>
     <row r="171" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B171" s="4"/>
+      <c r="B171" s="3"/>
     </row>
     <row r="172" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B172" s="4"/>
+      <c r="B172" s="3"/>
     </row>
     <row r="173" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B173" s="4"/>
+      <c r="B173" s="3"/>
     </row>
     <row r="174" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B174" s="4"/>
+      <c r="B174" s="3"/>
     </row>
     <row r="175" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B175" s="4"/>
+      <c r="B175" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Build unified Excel DD report
</commit_message>
<xml_diff>
--- a/Расчет_список.xlsx
+++ b/Расчет_список.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Users\Roman\Documents\DD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF4F1D7B-CA05-4A82-A362-B7B8665FA946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C12E7142-C825-41C0-AB63-1FA4A194D65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A77F7C32-41CE-594D-B64E-396197F2C882}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="84">
   <si>
     <t>Юнит</t>
   </si>
@@ -68,18 +68,12 @@
     <t>КАСКО</t>
   </si>
   <si>
-    <t>ИнтвестКопилка</t>
-  </si>
-  <si>
     <t xml:space="preserve">Развивающиеся </t>
   </si>
   <si>
     <t>СберСова</t>
   </si>
   <si>
-    <t>Залоговое страхование (корпоративное страхование)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Требуют внимания </t>
   </si>
   <si>
@@ -278,19 +272,34 @@
     <t>ОСАГО</t>
   </si>
   <si>
-    <t>сегмент</t>
-  </si>
-  <si>
     <t>SberPay Вжух</t>
   </si>
   <si>
     <t>Молодежь</t>
+  </si>
+  <si>
+    <t>ИнвестКопилка</t>
+  </si>
+  <si>
+    <t>Залоговое страхование (корпоративное)</t>
+  </si>
+  <si>
+    <t>Сегмент</t>
+  </si>
+  <si>
+    <t>Сценарии оплаты</t>
+  </si>
+  <si>
+    <t>СберСпасибо</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -347,7 +356,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
+        <bgColor theme="7" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
   </fills>
@@ -373,7 +382,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -383,15 +392,11 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -711,7 +716,7 @@
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="47.875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11" style="10"/>
+    <col min="4" max="4" width="11" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -722,7 +727,7 @@
       <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
@@ -740,15 +745,15 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D2" s="10">
+        <v>76</v>
+      </c>
+      <c r="D2" s="6">
         <v>0.62574257425742574</v>
       </c>
       <c r="E2" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" t="s">
         <v>7</v>
       </c>
     </row>
@@ -762,13 +767,13 @@
       <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="6">
         <v>0.62574257425742574</v>
       </c>
       <c r="E3" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -780,15 +785,15 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="10">
+        <v>79</v>
+      </c>
+      <c r="D4" s="6">
         <v>0.47640449438202248</v>
       </c>
       <c r="E4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -800,15 +805,15 @@
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="10">
-        <v>0.41396508728179554</v>
+        <v>10</v>
+      </c>
+      <c r="D5" s="6">
+        <v>0.47293447293447294</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -820,15 +825,15 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="10">
+        <v>80</v>
+      </c>
+      <c r="D6" s="6">
         <v>0.36082474226804123</v>
       </c>
       <c r="E6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
         <v>7</v>
       </c>
     </row>
@@ -840,15 +845,15 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="10">
+        <v>12</v>
+      </c>
+      <c r="D7" s="6">
         <v>0.46419753086419757</v>
       </c>
       <c r="E7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F7" t="s">
         <v>7</v>
       </c>
     </row>
@@ -860,15 +865,15 @@
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="10">
+        <v>13</v>
+      </c>
+      <c r="D8" s="6">
         <v>0.46236559139784944</v>
       </c>
       <c r="E8" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" t="s">
         <v>7</v>
       </c>
     </row>
@@ -880,15 +885,15 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="10">
+        <v>14</v>
+      </c>
+      <c r="D9" s="6">
         <v>0.39999999999999997</v>
       </c>
       <c r="E9" t="s">
-        <v>10</v>
-      </c>
-      <c r="F9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" t="s">
         <v>7</v>
       </c>
     </row>
@@ -900,15 +905,15 @@
         <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="10">
-        <v>0.44158415841584159</v>
+        <v>15</v>
+      </c>
+      <c r="D10" s="6">
+        <v>0.42178217821782182</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
-      </c>
-      <c r="F10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F10" t="s">
         <v>7</v>
       </c>
     </row>
@@ -920,15 +925,15 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="10">
+        <v>16</v>
+      </c>
+      <c r="D11" s="6">
         <v>0.47010309278350515</v>
       </c>
       <c r="E11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F11" t="s">
         <v>7</v>
       </c>
     </row>
@@ -940,15 +945,15 @@
         <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>19</v>
-      </c>
-      <c r="D12" s="10">
+        <v>17</v>
+      </c>
+      <c r="D12" s="6">
         <v>0.63505154639175254</v>
       </c>
       <c r="E12" t="s">
         <v>6</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" t="s">
         <v>7</v>
       </c>
     </row>
@@ -960,15 +965,15 @@
         <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="10">
+        <v>18</v>
+      </c>
+      <c r="D13" s="6">
         <v>0.53195876288659794</v>
       </c>
       <c r="E13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" t="s">
         <v>7</v>
       </c>
     </row>
@@ -980,15 +985,15 @@
         <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
-      </c>
-      <c r="D14" s="10">
+        <v>19</v>
+      </c>
+      <c r="D14" s="6">
         <v>0.60990099009900989</v>
       </c>
       <c r="E14" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1000,15 +1005,15 @@
         <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="10">
+        <v>20</v>
+      </c>
+      <c r="D15" s="6">
         <v>0.57029702970297036</v>
       </c>
       <c r="E15" t="s">
-        <v>10</v>
-      </c>
-      <c r="F15" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F15" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1020,15 +1025,15 @@
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>23</v>
-      </c>
-      <c r="D16" s="10">
+        <v>21</v>
+      </c>
+      <c r="D16" s="6">
         <v>0.38651685393258428</v>
       </c>
       <c r="E16" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1040,15 +1045,15 @@
         <v>5</v>
       </c>
       <c r="C17" t="s">
-        <v>24</v>
-      </c>
-      <c r="D17" s="10">
+        <v>22</v>
+      </c>
+      <c r="D17" s="6">
         <v>0.51546391752577314</v>
       </c>
       <c r="E17" t="s">
-        <v>10</v>
-      </c>
-      <c r="F17" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F17" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1060,15 +1065,15 @@
         <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>25</v>
-      </c>
-      <c r="D18" s="10">
+        <v>23</v>
+      </c>
+      <c r="D18" s="6">
         <v>0.59381443298969061</v>
       </c>
       <c r="E18" t="s">
-        <v>10</v>
-      </c>
-      <c r="F18" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F18" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1080,15 +1085,15 @@
         <v>5</v>
       </c>
       <c r="C19" t="s">
-        <v>26</v>
-      </c>
-      <c r="D19" s="10">
+        <v>24</v>
+      </c>
+      <c r="D19" s="6">
         <v>0.54491017964071853</v>
       </c>
       <c r="E19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F19" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F19" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1100,15 +1105,15 @@
         <v>5</v>
       </c>
       <c r="C20" t="s">
-        <v>27</v>
-      </c>
-      <c r="D20" s="10">
+        <v>25</v>
+      </c>
+      <c r="D20" s="6">
         <v>0.5388235294117647</v>
       </c>
       <c r="E20" t="s">
-        <v>10</v>
-      </c>
-      <c r="F20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F20" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1120,15 +1125,15 @@
         <v>5</v>
       </c>
       <c r="C21" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="10">
+        <v>26</v>
+      </c>
+      <c r="D21" s="6">
         <v>0.55730337078651682</v>
       </c>
       <c r="E21" t="s">
-        <v>10</v>
-      </c>
-      <c r="F21" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F21" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1140,15 +1145,15 @@
         <v>5</v>
       </c>
       <c r="C22" t="s">
-        <v>29</v>
-      </c>
-      <c r="D22" s="10">
+        <v>27</v>
+      </c>
+      <c r="D22" s="6">
         <v>0.2880886426592798</v>
       </c>
       <c r="E22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1157,18 +1162,18 @@
         <v>14</v>
       </c>
       <c r="B23" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C23" t="s">
-        <v>31</v>
-      </c>
-      <c r="D23" s="10">
-        <v>0.33980582524271846</v>
+        <v>29</v>
+      </c>
+      <c r="D23" s="6">
+        <v>0.39805825242718446</v>
       </c>
       <c r="E23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F23" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1177,18 +1182,18 @@
         <v>19</v>
       </c>
       <c r="B24" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" t="s">
         <v>30</v>
       </c>
-      <c r="C24" t="s">
-        <v>32</v>
-      </c>
-      <c r="D24" s="10">
+      <c r="D24" s="6">
         <v>0.60759493670886078</v>
       </c>
       <c r="E24" t="s">
         <v>6</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="F24" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1197,18 +1202,18 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C25" t="s">
-        <v>33</v>
-      </c>
-      <c r="D25" s="10">
-        <v>0.55089820359281438</v>
+        <v>31</v>
+      </c>
+      <c r="D25" s="6">
+        <v>0.42516268980477223</v>
       </c>
       <c r="E25" t="s">
-        <v>10</v>
-      </c>
-      <c r="F25" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F25" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1217,18 +1222,18 @@
         <v>29</v>
       </c>
       <c r="B26" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C26" t="s">
-        <v>34</v>
-      </c>
-      <c r="D26" s="10">
+        <v>32</v>
+      </c>
+      <c r="D26" s="6">
         <v>0.47524752475247523</v>
       </c>
       <c r="E26" t="s">
-        <v>10</v>
-      </c>
-      <c r="F26" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F26" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1237,18 +1242,18 @@
         <v>34</v>
       </c>
       <c r="B27" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C27" t="s">
-        <v>35</v>
-      </c>
-      <c r="D27" s="10">
+        <v>33</v>
+      </c>
+      <c r="D27" s="6">
         <v>0.55172413793103448</v>
       </c>
       <c r="E27" t="s">
-        <v>10</v>
-      </c>
-      <c r="F27" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F27" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1257,18 +1262,18 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C28" t="s">
-        <v>36</v>
-      </c>
-      <c r="D28" s="10">
+        <v>34</v>
+      </c>
+      <c r="D28" s="6">
         <v>0.5544554455445545</v>
       </c>
       <c r="E28" t="s">
-        <v>10</v>
-      </c>
-      <c r="F28" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F28" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1277,18 +1282,18 @@
         <v>223</v>
       </c>
       <c r="B29" t="s">
-        <v>30</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D29" s="10">
+        <v>28</v>
+      </c>
+      <c r="C29" t="s">
+        <v>35</v>
+      </c>
+      <c r="D29" s="6">
         <v>0.28817204301075267</v>
       </c>
       <c r="E29" t="s">
-        <v>13</v>
-      </c>
-      <c r="F29" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1297,18 +1302,18 @@
         <v>44</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C30" t="s">
-        <v>38</v>
-      </c>
-      <c r="D30" s="10">
+        <v>36</v>
+      </c>
+      <c r="D30" s="6">
         <v>0.76831683168316822</v>
       </c>
       <c r="E30" t="s">
         <v>6</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="F30" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1317,18 +1322,18 @@
         <v>49</v>
       </c>
       <c r="B31" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C31" t="s">
-        <v>39</v>
-      </c>
-      <c r="D31" s="10">
+        <v>37</v>
+      </c>
+      <c r="D31" s="6">
         <v>0.3827956989247312</v>
       </c>
       <c r="E31" t="s">
-        <v>13</v>
-      </c>
-      <c r="F31" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1337,18 +1342,18 @@
         <v>54</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C32" t="s">
-        <v>40</v>
-      </c>
-      <c r="D32" s="10">
+        <v>38</v>
+      </c>
+      <c r="D32" s="6">
         <v>0.34408602150537637</v>
       </c>
       <c r="E32" t="s">
-        <v>13</v>
-      </c>
-      <c r="F32" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1357,18 +1362,18 @@
         <v>181</v>
       </c>
       <c r="B33" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D33" s="10">
+        <v>40</v>
+      </c>
+      <c r="D33" s="6">
         <v>0.67010309278350511</v>
       </c>
       <c r="E33" t="s">
         <v>6</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="F33" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1377,18 +1382,18 @@
         <v>186</v>
       </c>
       <c r="B34" t="s">
+        <v>39</v>
+      </c>
+      <c r="C34" t="s">
         <v>41</v>
       </c>
-      <c r="C34" t="s">
-        <v>43</v>
-      </c>
-      <c r="D34" s="10">
+      <c r="D34" s="6">
         <v>0.6</v>
       </c>
       <c r="E34" t="s">
         <v>6</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="F34" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1397,18 +1402,18 @@
         <v>206</v>
       </c>
       <c r="B35" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C35" t="s">
-        <v>44</v>
-      </c>
-      <c r="D35" s="10">
+        <v>42</v>
+      </c>
+      <c r="D35" s="6">
         <v>0.73267326732673266</v>
       </c>
       <c r="E35" t="s">
         <v>6</v>
       </c>
-      <c r="F35" s="3" t="s">
+      <c r="F35" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1417,18 +1422,18 @@
         <v>217</v>
       </c>
       <c r="B36" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C36" t="s">
-        <v>46</v>
-      </c>
-      <c r="D36" s="10">
+        <v>44</v>
+      </c>
+      <c r="D36" s="6">
         <v>0.52861952861952854</v>
       </c>
       <c r="E36" t="s">
-        <v>10</v>
-      </c>
-      <c r="F36" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F36" s="7" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1436,19 +1441,19 @@
       <c r="A37">
         <v>229</v>
       </c>
-      <c r="B37" s="3" t="s">
-        <v>47</v>
+      <c r="B37" t="s">
+        <v>45</v>
       </c>
       <c r="C37" t="s">
-        <v>48</v>
-      </c>
-      <c r="D37" s="10">
+        <v>46</v>
+      </c>
+      <c r="D37" s="6">
         <v>0.57731958762886593</v>
       </c>
       <c r="E37" t="s">
-        <v>10</v>
-      </c>
-      <c r="F37" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F37" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1456,19 +1461,19 @@
       <c r="A38">
         <v>234</v>
       </c>
-      <c r="B38" s="3" t="s">
+      <c r="B38" t="s">
+        <v>45</v>
+      </c>
+      <c r="C38" t="s">
         <v>47</v>
       </c>
-      <c r="C38" t="s">
-        <v>49</v>
-      </c>
-      <c r="D38" s="10">
-        <v>0.56831683168316827</v>
+      <c r="D38" s="6">
+        <v>0.58415841584158412</v>
       </c>
       <c r="E38" t="s">
-        <v>10</v>
-      </c>
-      <c r="F38" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F38" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1476,179 +1481,179 @@
       <c r="A39">
         <v>239</v>
       </c>
-      <c r="B39" s="3" t="s">
-        <v>47</v>
+      <c r="B39" t="s">
+        <v>45</v>
       </c>
       <c r="C39" t="s">
+        <v>48</v>
+      </c>
+      <c r="D39" s="6">
+        <v>0.44950495049504952</v>
+      </c>
+      <c r="E39" t="s">
+        <v>9</v>
+      </c>
+      <c r="F39" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="8">
+        <v>13</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D40" s="9">
+        <v>0.55813953488372092</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F40" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="8">
+        <v>18</v>
+      </c>
+      <c r="B41" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D41" s="9">
+        <v>0.48091603053435117</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="8">
+        <v>23</v>
+      </c>
+      <c r="B42" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C42" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D39" s="10">
-        <v>0.44950495049504952</v>
-      </c>
-      <c r="E39" t="s">
-        <v>10</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="6">
-        <v>13</v>
-      </c>
-      <c r="B40" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C40" s="6" t="s">
+      <c r="D42" s="9">
+        <v>0.62287104622871048</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F42" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="8">
+        <v>28</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C43" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D40" s="11">
-        <v>0.58397932816537468</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F40" s="7" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="6">
-        <v>18</v>
-      </c>
-      <c r="B41" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C41" s="8" t="s">
+      <c r="D43" s="9">
+        <v>0.40203562340966925</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F43" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="D41" s="11">
-        <v>0.53180661577608146</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="6">
-        <v>23</v>
-      </c>
-      <c r="B42" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C42" s="8" t="s">
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="8">
+        <v>33</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C44" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D42" s="11">
-        <v>0.67153284671532842</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="6">
-        <v>28</v>
-      </c>
-      <c r="B43" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C43" s="8" t="s">
+      <c r="D44" s="9">
+        <v>0.55494505494505497</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F44" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="8">
+        <v>38</v>
+      </c>
+      <c r="B45" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C45" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="D43" s="11">
-        <v>0.49109414758269726</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="6">
-        <v>33</v>
-      </c>
-      <c r="B44" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C44" s="8" t="s">
+      <c r="D45" s="9">
+        <v>0.52247191011235961</v>
+      </c>
+      <c r="E45" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F45" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="8">
+        <v>43</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C46" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="D44" s="11">
-        <v>0.59890109890109888</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="6">
-        <v>38</v>
-      </c>
-      <c r="B45" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C45" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="D45" s="11">
-        <v>0.6797752808988764</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="F45" s="7" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="6">
-        <v>43</v>
-      </c>
-      <c r="B46" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="C46" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D46" s="11">
-        <v>0.4438202247191011</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="F46" s="7" t="s">
-        <v>79</v>
+      <c r="D46" s="9">
+        <v>0.398876404494382</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F46" s="8" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>260</v>
       </c>
-      <c r="B47" s="3" t="s">
-        <v>57</v>
+      <c r="B47" t="s">
+        <v>55</v>
       </c>
       <c r="C47" t="s">
-        <v>58</v>
-      </c>
-      <c r="D47" s="10">
+        <v>56</v>
+      </c>
+      <c r="D47" s="6">
         <v>0.34457831325301208</v>
       </c>
       <c r="E47" t="s">
-        <v>13</v>
-      </c>
-      <c r="F47" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F47" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1656,19 +1661,19 @@
       <c r="A48">
         <v>280</v>
       </c>
-      <c r="B48" s="3" t="s">
+      <c r="B48" t="s">
+        <v>55</v>
+      </c>
+      <c r="C48" t="s">
         <v>57</v>
       </c>
-      <c r="C48" t="s">
-        <v>59</v>
-      </c>
-      <c r="D48" s="10">
+      <c r="D48" s="6">
         <v>0.27586206896551724</v>
       </c>
       <c r="E48" t="s">
-        <v>13</v>
-      </c>
-      <c r="F48" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F48" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1676,19 +1681,19 @@
       <c r="A49">
         <v>285</v>
       </c>
-      <c r="B49" s="3" t="s">
-        <v>57</v>
+      <c r="B49" t="s">
+        <v>55</v>
       </c>
       <c r="C49" t="s">
-        <v>60</v>
-      </c>
-      <c r="D49" s="10">
+        <v>58</v>
+      </c>
+      <c r="D49" s="6">
         <v>0.24</v>
       </c>
       <c r="E49" t="s">
-        <v>13</v>
-      </c>
-      <c r="F49" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F49" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1696,19 +1701,19 @@
       <c r="A50">
         <v>290</v>
       </c>
-      <c r="B50" s="3" t="s">
-        <v>57</v>
+      <c r="B50" t="s">
+        <v>55</v>
       </c>
       <c r="C50" t="s">
-        <v>61</v>
-      </c>
-      <c r="D50" s="10">
+        <v>59</v>
+      </c>
+      <c r="D50" s="6">
         <v>0.35632183908045978</v>
       </c>
       <c r="E50" t="s">
-        <v>13</v>
-      </c>
-      <c r="F50" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F50" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1716,19 +1721,19 @@
       <c r="A51">
         <v>300</v>
       </c>
-      <c r="B51" s="3" t="s">
-        <v>57</v>
+      <c r="B51" t="s">
+        <v>55</v>
       </c>
       <c r="C51" t="s">
-        <v>62</v>
-      </c>
-      <c r="D51" s="10">
+        <v>60</v>
+      </c>
+      <c r="D51" s="6">
         <v>0.58969072164948455</v>
       </c>
       <c r="E51" t="s">
-        <v>10</v>
-      </c>
-      <c r="F51" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F51" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1736,19 +1741,19 @@
       <c r="A52">
         <v>315</v>
       </c>
-      <c r="B52" s="3" t="s">
-        <v>57</v>
+      <c r="B52" t="s">
+        <v>55</v>
       </c>
       <c r="C52" t="s">
-        <v>63</v>
-      </c>
-      <c r="D52" s="10">
+        <v>61</v>
+      </c>
+      <c r="D52" s="6">
         <v>0.37362637362637363</v>
       </c>
       <c r="E52" t="s">
-        <v>13</v>
-      </c>
-      <c r="F52" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F52" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1756,19 +1761,19 @@
       <c r="A53">
         <v>320</v>
       </c>
-      <c r="B53" s="3" t="s">
-        <v>57</v>
+      <c r="B53" t="s">
+        <v>55</v>
       </c>
       <c r="C53" t="s">
-        <v>64</v>
-      </c>
-      <c r="D53" s="10">
+        <v>62</v>
+      </c>
+      <c r="D53" s="6">
         <v>0.36831683168316837</v>
       </c>
       <c r="E53" t="s">
-        <v>13</v>
-      </c>
-      <c r="F53" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F53" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1776,19 +1781,19 @@
       <c r="A54">
         <v>325</v>
       </c>
-      <c r="B54" s="3" t="s">
-        <v>57</v>
+      <c r="B54" t="s">
+        <v>55</v>
       </c>
       <c r="C54" t="s">
-        <v>65</v>
-      </c>
-      <c r="D54" s="10">
+        <v>63</v>
+      </c>
+      <c r="D54" s="6">
         <v>0.68247422680412373</v>
       </c>
       <c r="E54" t="s">
         <v>6</v>
       </c>
-      <c r="F54" s="3" t="s">
+      <c r="F54" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1796,19 +1801,19 @@
       <c r="A55">
         <v>330</v>
       </c>
-      <c r="B55" s="3" t="s">
-        <v>57</v>
+      <c r="B55" t="s">
+        <v>55</v>
       </c>
       <c r="C55" t="s">
-        <v>66</v>
-      </c>
-      <c r="D55" s="10">
+        <v>64</v>
+      </c>
+      <c r="D55" s="6">
         <v>0.37354988399071926</v>
       </c>
       <c r="E55" t="s">
-        <v>13</v>
-      </c>
-      <c r="F55" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F55" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1816,19 +1821,19 @@
       <c r="A56">
         <v>335</v>
       </c>
-      <c r="B56" s="3" t="s">
-        <v>57</v>
+      <c r="B56" t="s">
+        <v>55</v>
       </c>
       <c r="C56" t="s">
-        <v>67</v>
-      </c>
-      <c r="D56" s="10">
+        <v>65</v>
+      </c>
+      <c r="D56" s="6">
         <v>0.65822784810126578</v>
       </c>
       <c r="E56" t="s">
         <v>6</v>
       </c>
-      <c r="F56" s="3" t="s">
+      <c r="F56" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1836,19 +1841,19 @@
       <c r="A57">
         <v>340</v>
       </c>
-      <c r="B57" s="3" t="s">
-        <v>57</v>
+      <c r="B57" t="s">
+        <v>55</v>
       </c>
       <c r="C57" t="s">
-        <v>68</v>
-      </c>
-      <c r="D57" s="10">
+        <v>66</v>
+      </c>
+      <c r="D57" s="6">
         <v>0.62650602409638556</v>
       </c>
       <c r="E57" t="s">
         <v>6</v>
       </c>
-      <c r="F57" s="3" t="s">
+      <c r="F57" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1856,19 +1861,19 @@
       <c r="A58">
         <v>345</v>
       </c>
-      <c r="B58" s="3" t="s">
-        <v>57</v>
+      <c r="B58" t="s">
+        <v>55</v>
       </c>
       <c r="C58" t="s">
-        <v>69</v>
-      </c>
-      <c r="D58" s="10">
+        <v>67</v>
+      </c>
+      <c r="D58" s="6">
         <v>0.55643564356435649</v>
       </c>
       <c r="E58" t="s">
-        <v>10</v>
-      </c>
-      <c r="F58" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F58" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1876,19 +1881,19 @@
       <c r="A59">
         <v>350</v>
       </c>
-      <c r="B59" s="3" t="s">
-        <v>57</v>
+      <c r="B59" t="s">
+        <v>55</v>
       </c>
       <c r="C59" t="s">
-        <v>70</v>
-      </c>
-      <c r="D59" s="10">
+        <v>68</v>
+      </c>
+      <c r="D59" s="6">
         <v>0.77367205542725181</v>
       </c>
       <c r="E59" t="s">
         <v>6</v>
       </c>
-      <c r="F59" s="3" t="s">
+      <c r="F59" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1896,19 +1901,19 @@
       <c r="A60">
         <v>355</v>
       </c>
-      <c r="B60" s="3" t="s">
-        <v>57</v>
+      <c r="B60" t="s">
+        <v>55</v>
       </c>
       <c r="C60" t="s">
-        <v>71</v>
-      </c>
-      <c r="D60" s="10">
+        <v>69</v>
+      </c>
+      <c r="D60" s="6">
         <v>0.36263736263736263</v>
       </c>
       <c r="E60" t="s">
-        <v>13</v>
-      </c>
-      <c r="F60" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F60" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1916,19 +1921,19 @@
       <c r="A61">
         <v>360</v>
       </c>
-      <c r="B61" s="3" t="s">
-        <v>57</v>
+      <c r="B61" t="s">
+        <v>55</v>
       </c>
       <c r="C61" t="s">
-        <v>64</v>
-      </c>
-      <c r="D61" s="10">
-        <v>0.45940594059405937</v>
+        <v>82</v>
+      </c>
+      <c r="D61" s="6">
+        <v>0.47524752475247523</v>
       </c>
       <c r="E61" t="s">
-        <v>10</v>
-      </c>
-      <c r="F61" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F61" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1936,19 +1941,19 @@
       <c r="A62">
         <v>365</v>
       </c>
-      <c r="B62" s="3" t="s">
-        <v>57</v>
+      <c r="B62" t="s">
+        <v>55</v>
       </c>
       <c r="C62" t="s">
-        <v>72</v>
-      </c>
-      <c r="D62" s="10">
+        <v>70</v>
+      </c>
+      <c r="D62" s="6">
         <v>0.37349397590361444</v>
       </c>
       <c r="E62" t="s">
-        <v>13</v>
-      </c>
-      <c r="F62" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F62" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1956,19 +1961,19 @@
       <c r="A63">
         <v>370</v>
       </c>
-      <c r="B63" s="3" t="s">
-        <v>57</v>
+      <c r="B63" t="s">
+        <v>55</v>
       </c>
       <c r="C63" t="s">
-        <v>73</v>
-      </c>
-      <c r="D63" s="10">
+        <v>71</v>
+      </c>
+      <c r="D63" s="6">
         <v>0.41445783132530117</v>
       </c>
       <c r="E63" t="s">
-        <v>10</v>
-      </c>
-      <c r="F63" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F63" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1976,19 +1981,19 @@
       <c r="A64">
         <v>375</v>
       </c>
-      <c r="B64" s="3" t="s">
-        <v>57</v>
+      <c r="B64" t="s">
+        <v>55</v>
       </c>
       <c r="C64" t="s">
-        <v>80</v>
-      </c>
-      <c r="D64" s="10">
+        <v>77</v>
+      </c>
+      <c r="D64" s="6">
         <v>0.4206896551724138</v>
       </c>
       <c r="E64" t="s">
-        <v>10</v>
-      </c>
-      <c r="F64" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F64" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1996,19 +2001,19 @@
       <c r="A65">
         <v>380</v>
       </c>
-      <c r="B65" s="3" t="s">
-        <v>57</v>
+      <c r="B65" t="s">
+        <v>55</v>
       </c>
       <c r="C65" t="s">
-        <v>74</v>
-      </c>
-      <c r="D65" s="10">
+        <v>72</v>
+      </c>
+      <c r="D65" s="6">
         <v>0.33195876288659798</v>
       </c>
       <c r="E65" t="s">
-        <v>13</v>
-      </c>
-      <c r="F65" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F65" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2016,19 +2021,19 @@
       <c r="A66">
         <v>390</v>
       </c>
-      <c r="B66" s="3" t="s">
-        <v>57</v>
+      <c r="B66" t="s">
+        <v>55</v>
       </c>
       <c r="C66" t="s">
-        <v>75</v>
-      </c>
-      <c r="D66" s="10">
+        <v>73</v>
+      </c>
+      <c r="D66" s="6">
         <v>0.3935483870967742</v>
       </c>
       <c r="E66" t="s">
-        <v>13</v>
-      </c>
-      <c r="F66" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F66" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2036,19 +2041,19 @@
       <c r="A67">
         <v>405</v>
       </c>
-      <c r="B67" s="3" t="s">
-        <v>57</v>
+      <c r="B67" t="s">
+        <v>55</v>
       </c>
       <c r="C67" t="s">
-        <v>76</v>
-      </c>
-      <c r="D67" s="10">
+        <v>74</v>
+      </c>
+      <c r="D67" s="6">
         <v>0.33806146572104023</v>
       </c>
       <c r="E67" t="s">
-        <v>13</v>
-      </c>
-      <c r="F67" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F67" t="s">
         <v>7</v>
       </c>
     </row>
@@ -2056,24 +2061,41 @@
       <c r="A68">
         <v>410</v>
       </c>
-      <c r="B68" s="3" t="s">
-        <v>57</v>
+      <c r="B68" t="s">
+        <v>55</v>
       </c>
       <c r="C68" t="s">
-        <v>77</v>
-      </c>
-      <c r="D68" s="10">
+        <v>75</v>
+      </c>
+      <c r="D68" s="6">
         <v>0.39958592132505177</v>
       </c>
       <c r="E68" t="s">
-        <v>13</v>
-      </c>
-      <c r="F68" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F68" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B69" s="3"/>
+      <c r="A69">
+        <v>420</v>
+      </c>
+      <c r="B69" t="s">
+        <v>45</v>
+      </c>
+      <c r="C69" t="s">
+        <v>83</v>
+      </c>
+      <c r="D69" s="6">
+        <v>0.68493150684931503</v>
+      </c>
+      <c r="E69" t="s">
+        <v>6</v>
+      </c>
+      <c r="F69" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B70" s="3"/>

</xml_diff>